<commit_message>
add data dict to math ela grad sheet
</commit_message>
<xml_diff>
--- a/products/edde/resources/quality_of_life/education_math_ela_grad.xlsx
+++ b/products/edde/resources/quality_of_life/education_math_ela_grad.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexrichey/dev/data-engineering-de2/products/edde/resources/quality_of_life/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2682E5-0011-B941-A09A-93D6EA9085B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151611D3-DA79-8C41-9522-0C2EE74EB311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10520" yWindow="-27900" windowWidth="37100" windowHeight="26400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Data Dictionary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="638">
   <si>
     <t>NTA Code</t>
   </si>
@@ -1675,6 +1676,282 @@
   <si>
     <t>Miller Field</t>
   </si>
+  <si>
+    <t>varname</t>
+  </si>
+  <si>
+    <t>varlabel</t>
+  </si>
+  <si>
+    <t>ntacode</t>
+  </si>
+  <si>
+    <t>ntaname</t>
+  </si>
+  <si>
+    <t>tot_ela_tested</t>
+  </si>
+  <si>
+    <t>ela_tested_Asian</t>
+  </si>
+  <si>
+    <t>ela_tested_Black</t>
+  </si>
+  <si>
+    <t>ela_tested_Hispanic</t>
+  </si>
+  <si>
+    <t>ela_tested_White</t>
+  </si>
+  <si>
+    <t>ela_tested_Multi_Racial</t>
+  </si>
+  <si>
+    <t>ela_tested_Native_American</t>
+  </si>
+  <si>
+    <t>ela_tested_Race_Missing</t>
+  </si>
+  <si>
+    <t>tot_ela_prof</t>
+  </si>
+  <si>
+    <t>ela_prof_Asian</t>
+  </si>
+  <si>
+    <t>ela_prof_Black</t>
+  </si>
+  <si>
+    <t>ela_prof_Hispanic</t>
+  </si>
+  <si>
+    <t>ela_prof_White</t>
+  </si>
+  <si>
+    <t>ela_prof_Multi_Racial</t>
+  </si>
+  <si>
+    <t>ela_prof_Native_American</t>
+  </si>
+  <si>
+    <t>ela_prof_Race_Missing</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof_Asian</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof_Black</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof_Hispanic</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof_White</t>
+  </si>
+  <si>
+    <t>perct_tot_ela_prof_MultiRacial</t>
+  </si>
+  <si>
+    <t>perct_totela_prof_NativeAmerican</t>
+  </si>
+  <si>
+    <t>perct_totela_prof_RaceMissing</t>
+  </si>
+  <si>
+    <t>tot_math_tested</t>
+  </si>
+  <si>
+    <t>math_tested_Asian</t>
+  </si>
+  <si>
+    <t>math_tested_Black</t>
+  </si>
+  <si>
+    <t>math_tested_Hispanic</t>
+  </si>
+  <si>
+    <t>math_tested_White</t>
+  </si>
+  <si>
+    <t>math_tested_Multi_Racial</t>
+  </si>
+  <si>
+    <t>math_tested_Native_American</t>
+  </si>
+  <si>
+    <t>math_tested_Race_Missing</t>
+  </si>
+  <si>
+    <t>tot_math_prof</t>
+  </si>
+  <si>
+    <t>math_prof_Asian</t>
+  </si>
+  <si>
+    <t>math_prof_Black</t>
+  </si>
+  <si>
+    <t>math_prof_Hispanic</t>
+  </si>
+  <si>
+    <t>math_prof_White</t>
+  </si>
+  <si>
+    <t>math_prof_Multi_Racial</t>
+  </si>
+  <si>
+    <t>math_prof_Native_American</t>
+  </si>
+  <si>
+    <t>math_prof_Race_Missing</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof_Asian</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof_Black</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof_Hispanic</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof_White</t>
+  </si>
+  <si>
+    <t>perct_tot_math_prof_MultiRacial</t>
+  </si>
+  <si>
+    <t>perct_totmathprof_NativeAmerican</t>
+  </si>
+  <si>
+    <t>perct_totmath_prof_RaceMissing</t>
+  </si>
+  <si>
+    <t>tot_grad_cohort</t>
+  </si>
+  <si>
+    <t>cohort_Asian</t>
+  </si>
+  <si>
+    <t>cohort_Black</t>
+  </si>
+  <si>
+    <t>cohort_Hispanic</t>
+  </si>
+  <si>
+    <t>cohort_White</t>
+  </si>
+  <si>
+    <t>cohort_Multi_Racial</t>
+  </si>
+  <si>
+    <t>cohort_Native_American</t>
+  </si>
+  <si>
+    <t>cohort_Race_Missing</t>
+  </si>
+  <si>
+    <t>tot_grads</t>
+  </si>
+  <si>
+    <t>grad_Asian</t>
+  </si>
+  <si>
+    <t>grad_Black</t>
+  </si>
+  <si>
+    <t>grad_Hispanic</t>
+  </si>
+  <si>
+    <t>grad_White</t>
+  </si>
+  <si>
+    <t>grad_Multi_Racial</t>
+  </si>
+  <si>
+    <t>grad_Native_American</t>
+  </si>
+  <si>
+    <t>grad_Race_Missing</t>
+  </si>
+  <si>
+    <t>perct_tot_grads</t>
+  </si>
+  <si>
+    <t>perct_tot_grads_Asian</t>
+  </si>
+  <si>
+    <t>perct_tot_grads_Black</t>
+  </si>
+  <si>
+    <t>perct_tot_grads_Hispanic</t>
+  </si>
+  <si>
+    <t>perct_tot_grads_White</t>
+  </si>
+  <si>
+    <t>perct_tot_grads_MultiRacial</t>
+  </si>
+  <si>
+    <t>perct_totgrads_NativeAmerican</t>
+  </si>
+  <si>
+    <t>perct_totgrads_RaceMissing</t>
+  </si>
+  <si>
+    <t>tot_dropouts</t>
+  </si>
+  <si>
+    <t>dropout_Asian</t>
+  </si>
+  <si>
+    <t>dropout_Black</t>
+  </si>
+  <si>
+    <t>dropout_Hispanic</t>
+  </si>
+  <si>
+    <t>dropout_White</t>
+  </si>
+  <si>
+    <t>dropout_Multi_Racial</t>
+  </si>
+  <si>
+    <t>dropout_Native_American</t>
+  </si>
+  <si>
+    <t>dropout_Race_Missing</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_Asian</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_Black</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_Hispanic</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_White</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_MultiRacial</t>
+  </si>
+  <si>
+    <t>perct_totdropoutsNativeAmerican</t>
+  </si>
+  <si>
+    <t>perct_tot_dropouts_RaceMissing</t>
+  </si>
 </sst>
 </file>
 
@@ -1683,10 +1960,15 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1709,13 +1991,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -62973,13 +63256,757 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245957A6-83C6-4047-BEEB-9BCFBF35FC29}">
+  <dimension ref="A1:B91"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.33203125" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>599</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>604</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="4" t="s">
+        <v>620</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="4" t="s">
+        <v>621</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="4" t="s">
+        <v>625</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="4" t="s">
+        <v>626</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3d51228c-8aff-4099-8ffe-73dfbb04b9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -63224,20 +64251,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3d51228c-8aff-4099-8ffe-73dfbb04b9a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F818B31-833F-4D09-A8A4-CCD4C8D2B0CC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8197899-894F-4860-BD07-07E70E5AF6AE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3d51228c-8aff-4099-8ffe-73dfbb04b9a4"/>
+    <ds:schemaRef ds:uri="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -63262,12 +64290,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8197899-894F-4860-BD07-07E70E5AF6AE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F818B31-833F-4D09-A8A4-CCD4C8D2B0CC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3d51228c-8aff-4099-8ffe-73dfbb04b9a4"/>
-    <ds:schemaRef ds:uri="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>